<commit_message>
Second commit with completed websites and partly implemented output excel logic.
</commit_message>
<xml_diff>
--- a/Data/Config.xlsx
+++ b/Data/Config.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\VedantVaibhavGham\Documents\UiPath\Dermalogica_Modern_Performer\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{59D4000B-598C-4BE6-9732-05FFEB307EA5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{30D9AC5D-72D8-4F6F-A2B1-2002A7337B84}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -663,7 +663,7 @@
       <c r="A7" t="s">
         <v>44</v>
       </c>
-      <c r="B7" t="s">
+      <c r="B7" s="5" t="s">
         <v>45</v>
       </c>
     </row>
@@ -671,7 +671,7 @@
       <c r="A8" t="s">
         <v>46</v>
       </c>
-      <c r="B8" t="s">
+      <c r="B8" s="5" t="s">
         <v>47</v>
       </c>
     </row>
@@ -687,7 +687,7 @@
       <c r="A10" t="s">
         <v>50</v>
       </c>
-      <c r="B10" t="s">
+      <c r="B10" s="5" t="s">
         <v>51</v>
       </c>
     </row>
@@ -695,7 +695,7 @@
       <c r="A11" t="s">
         <v>52</v>
       </c>
-      <c r="B11" t="s">
+      <c r="B11" s="5" t="s">
         <v>53</v>
       </c>
     </row>
@@ -703,7 +703,7 @@
       <c r="A12" t="s">
         <v>54</v>
       </c>
-      <c r="B12" t="s">
+      <c r="B12" s="5" t="s">
         <v>55</v>
       </c>
     </row>
@@ -711,7 +711,7 @@
       <c r="A13" t="s">
         <v>56</v>
       </c>
-      <c r="B13" t="s">
+      <c r="B13" s="5" t="s">
         <v>57</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Second last commit with all running websites, and exception in derma france.
</commit_message>
<xml_diff>
--- a/Data/Config.xlsx
+++ b/Data/Config.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\VedantVaibhavGham\Documents\UiPath\Dermalogica_Modern_Performer\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{30D9AC5D-72D8-4F6F-A2B1-2002A7337B84}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{477D1F42-0EA8-4810-84BE-1DF284A2661B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="64" uniqueCount="60">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="82" uniqueCount="78">
   <si>
     <t>Name</t>
   </si>
@@ -205,6 +205,60 @@
   </si>
   <si>
     <t>Shared</t>
+  </si>
+  <si>
+    <t>OutputReportPath</t>
+  </si>
+  <si>
+    <t>SheetName</t>
+  </si>
+  <si>
+    <t>Dermalogica Output Report</t>
+  </si>
+  <si>
+    <t>C:\Users\VedantVaibhavGham\Documents\UiPath\Dermalogica_Modern_Performer\Data\Output\OutputReport.xlsx</t>
+  </si>
+  <si>
+    <t>EndMailBody</t>
+  </si>
+  <si>
+    <t>Performer process completed for Dermalogica Modern Performer Process.</t>
+  </si>
+  <si>
+    <t>EndMailSubject</t>
+  </si>
+  <si>
+    <t>End Mail for Dermalogica Performer</t>
+  </si>
+  <si>
+    <t>ToField</t>
+  </si>
+  <si>
+    <t>Vedant.Gham@accelirate.com</t>
+  </si>
+  <si>
+    <t>StartMailBody</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Starting the Dermalogica Modern Performer </t>
+  </si>
+  <si>
+    <t>StartMailSubject</t>
+  </si>
+  <si>
+    <t>Start of Dermalogica Modern Performer</t>
+  </si>
+  <si>
+    <t>CurrentDateTime</t>
+  </si>
+  <si>
+    <t>dd-MM-yyyy HH:mm:ss</t>
+  </si>
+  <si>
+    <t>ProcessName</t>
+  </si>
+  <si>
+    <t>Dermalogica Performer</t>
   </si>
 </sst>
 </file>
@@ -663,7 +717,7 @@
       <c r="A7" t="s">
         <v>44</v>
       </c>
-      <c r="B7" s="5" t="s">
+      <c r="B7" t="s">
         <v>45</v>
       </c>
     </row>
@@ -671,7 +725,7 @@
       <c r="A8" t="s">
         <v>46</v>
       </c>
-      <c r="B8" s="5" t="s">
+      <c r="B8" t="s">
         <v>47</v>
       </c>
     </row>
@@ -679,7 +733,7 @@
       <c r="A9" t="s">
         <v>48</v>
       </c>
-      <c r="B9" s="5" t="s">
+      <c r="B9" t="s">
         <v>49</v>
       </c>
     </row>
@@ -687,7 +741,7 @@
       <c r="A10" t="s">
         <v>50</v>
       </c>
-      <c r="B10" s="5" t="s">
+      <c r="B10" t="s">
         <v>51</v>
       </c>
     </row>
@@ -695,7 +749,7 @@
       <c r="A11" t="s">
         <v>52</v>
       </c>
-      <c r="B11" s="5" t="s">
+      <c r="B11" t="s">
         <v>53</v>
       </c>
     </row>
@@ -703,7 +757,7 @@
       <c r="A12" t="s">
         <v>54</v>
       </c>
-      <c r="B12" s="5" t="s">
+      <c r="B12" t="s">
         <v>55</v>
       </c>
     </row>
@@ -711,29 +765,92 @@
       <c r="A13" t="s">
         <v>56</v>
       </c>
-      <c r="B13" s="5" t="s">
+      <c r="B13" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="14" spans="1:26" ht="14.25" customHeight="1"/>
-    <row r="15" spans="1:26" ht="14.25" customHeight="1"/>
-    <row r="16" spans="1:26" ht="14.25" customHeight="1"/>
-    <row r="17" ht="14.25" customHeight="1"/>
-    <row r="18" ht="14.25" customHeight="1"/>
-    <row r="19" ht="14.25" customHeight="1"/>
-    <row r="20" ht="14.25" customHeight="1"/>
-    <row r="21" ht="14.25" customHeight="1"/>
-    <row r="22" ht="14.25" customHeight="1"/>
-    <row r="23" ht="14.25" customHeight="1"/>
-    <row r="24" ht="14.25" customHeight="1"/>
-    <row r="25" ht="14.25" customHeight="1"/>
-    <row r="26" ht="14.25" customHeight="1"/>
-    <row r="27" ht="14.25" customHeight="1"/>
-    <row r="28" ht="14.25" customHeight="1"/>
-    <row r="29" ht="14.25" customHeight="1"/>
-    <row r="30" ht="14.25" customHeight="1"/>
-    <row r="31" ht="14.25" customHeight="1"/>
-    <row r="32" ht="14.25" customHeight="1"/>
+    <row r="14" spans="1:26" ht="14.25" customHeight="1">
+      <c r="A14" t="s">
+        <v>60</v>
+      </c>
+      <c r="B14" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="15" spans="1:26" ht="14.25" customHeight="1">
+      <c r="A15" t="s">
+        <v>61</v>
+      </c>
+      <c r="B15" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="16" spans="1:26" ht="14.25" customHeight="1">
+      <c r="A16" t="s">
+        <v>64</v>
+      </c>
+      <c r="B16" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" ht="14.25" customHeight="1">
+      <c r="A17" t="s">
+        <v>66</v>
+      </c>
+      <c r="B17" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" ht="14.25" customHeight="1">
+      <c r="A18" t="s">
+        <v>68</v>
+      </c>
+      <c r="B18" s="5" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" ht="14.25" customHeight="1">
+      <c r="A19" t="s">
+        <v>70</v>
+      </c>
+      <c r="B19" s="5" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" ht="14.25" customHeight="1">
+      <c r="A20" t="s">
+        <v>72</v>
+      </c>
+      <c r="B20" s="5" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" ht="14.25" customHeight="1">
+      <c r="A21" t="s">
+        <v>74</v>
+      </c>
+      <c r="B21" s="5" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" ht="14.25" customHeight="1">
+      <c r="A22" t="s">
+        <v>76</v>
+      </c>
+      <c r="B22" s="5" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" ht="14.25" customHeight="1"/>
+    <row r="24" spans="1:2" ht="14.25" customHeight="1"/>
+    <row r="25" spans="1:2" ht="14.25" customHeight="1"/>
+    <row r="26" spans="1:2" ht="14.25" customHeight="1"/>
+    <row r="27" spans="1:2" ht="14.25" customHeight="1"/>
+    <row r="28" spans="1:2" ht="14.25" customHeight="1"/>
+    <row r="29" spans="1:2" ht="14.25" customHeight="1"/>
+    <row r="30" spans="1:2" ht="14.25" customHeight="1"/>
+    <row r="31" spans="1:2" ht="14.25" customHeight="1"/>
+    <row r="32" spans="1:2" ht="14.25" customHeight="1"/>
     <row r="33" ht="14.25" customHeight="1"/>
     <row r="34" ht="14.25" customHeight="1"/>
     <row r="35" ht="14.25" customHeight="1"/>

</xml_diff>